<commit_message>
Audit workbook: dropdowns from a hidden list sheet, passage-number dropdown, input hints
</commit_message>
<xml_diff>
--- a/annotation/v04_miss_audit/miss_audit_v04.xlsx
+++ b/annotation/v04_miss_audit/miss_audit_v04.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screen2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4992,15 +4993,14 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="I2:I101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"yes,no,unsure"</formula1>
+    <dataValidation sqref="I2:I101" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Please choose a value from the list." promptTitle="Select" prompt="Choose yes / no / unsure" type="list">
+      <formula1>Lists!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"yes,no"</formula1>
+    <dataValidation sqref="J2:J101" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Please choose a value from the list." promptTitle="Select" prompt="If A = yes: choose the passage number 1-5" type="list">
+      <formula1>Lists!$C$1:$C$5</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
-      <formula1>1</formula1>
-      <formula2>5</formula2>
+    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Please choose a value from the list." promptTitle="Select" prompt="If A = yes: choose yes / no" type="list">
+      <formula1>Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7670,13 +7670,77 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"yes,no,unsure"</formula1>
+    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Please choose a value from the list." promptTitle="Select" prompt="Choose yes / no / unsure" type="list">
+      <formula1>Lists!$A$1:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"yes,no"</formula1>
+    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Please choose a value from the list." promptTitle="Select" prompt="If C = yes and EM = 0: choose yes / no" type="list">
+      <formula1>Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>unsure</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>